<commit_message>
Lernen bei Tabelllen eingabe und verbesserung der Abfrage
</commit_message>
<xml_diff>
--- a/Tabellen/Anatomie 1-Muskeln Detail-Gesäß-Gluteus.xlsx
+++ b/Tabellen/Anatomie 1-Muskeln Detail-Gesäß-Gluteus.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -61,35 +61,7 @@
     <t xml:space="preserve">Trochanter major Os Femoris</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Gesamt: Abduktion; Gesamt: Stabil Frontalebene; vordere Teil: Flexion; vordere Teil: Innenrotation; hintere Teil: Extension; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">hintere Teil:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Außenrotation</t>
-    </r>
+    <t xml:space="preserve">Gesamt: Abduktion; Gesamt: Stabil Frontalebene; vordere Teil: Flexion; vordere Teil: Innenrotation; hintere Teil: Extension; hintere Teil: Außenrotation</t>
   </si>
   <si>
     <t xml:space="preserve">N. gluteus superior L4–S1</t>
@@ -101,56 +73,6 @@
     <t xml:space="preserve">Facies glutea Os Ilium</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Abduktion; Stabil Frontalebene; vordere Teil: Flexion; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">vordere Teil:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Innenrotation; hintere Teil: Extension; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">hintere Teil:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Außenrotation</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">M. Tensor fasciae latae</t>
   </si>
   <si>
@@ -160,7 +82,7 @@
     <t xml:space="preserve">Tractus iliotibialis</t>
   </si>
   <si>
-    <t xml:space="preserve">spannt Fascia lata; Abduktion; Flexion; Innenrotation</t>
+    <t xml:space="preserve">Gesamt: spannt Fascia lata; Gesamt: Abduktion; Gesamt: Flexion; Gesamt: Innenrotation</t>
   </si>
 </sst>
 </file>
@@ -170,7 +92,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,12 +114,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -266,7 +182,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -464,7 +380,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="32.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.66"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="11.55"/>
@@ -532,24 +448,24 @@
         <v>12</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>14</v>

</xml_diff>